<commit_message>
Actualización automática historial PIB
</commit_message>
<xml_diff>
--- a/monitoreo_pib.xlsx
+++ b/monitoreo_pib.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,6 +458,120 @@
         <is>
           <t>Variacion (%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:32:39</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>XII</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>31866425.5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>31871088.6</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>4663.10000000149</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.01463326974028352</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:32:39</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>XII</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>33506846.9</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>33582899.3</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>76052.39999999851</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2269756991070339</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:32:39</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>XII</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>35255452.9</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>35301585.1</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>46132.20000000298</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1308512476945176</v>
       </c>
     </row>
   </sheetData>
@@ -471,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +609,18 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>Sin cambios</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-12 20:32:40</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cambios detectados (3)</t>
         </is>
       </c>
     </row>

</xml_diff>